<commit_message>
chore(i18n): Sync autoPreparing phase keys to translation sheet
Add syncActivity.phases.autoPreparingTitle and autoPreparingSubtitle
to docs/localization/mobile-i18n.xlsx so the translation sheet stays
aligned with the JSON locale files.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/localization/mobile-i18n.xlsx
+++ b/docs/localization/mobile-i18n.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F485"/>
+  <dimension ref="A1:F487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2999,7 +2999,6 @@
           <t>summary.unitCount</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>个</t>
@@ -7392,7 +7391,6 @@
           <t>cards.statsUnit</t>
         </is>
       </c>
-      <c r="D217" t="inlineStr"/>
       <c r="E217" t="inlineStr">
         <is>
           <t>个</t>
@@ -14007,27 +14005,27 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>syncActivity.phases.defaultTitle</t>
+          <t>syncActivity.phases.autoPreparingSubtitle</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>phases.defaultTitle</t>
+          <t>phases.autoPreparingSubtitle</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Preparing...</t>
+          <t>Preparing to scan for new photos</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>准备中…</t>
+          <t>即将开始扫描新照片</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t>準備中…</t>
+          <t>即將開始掃描新照片</t>
         </is>
       </c>
     </row>
@@ -14039,27 +14037,27 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>syncActivity.phases.discoveringSubtitleSearching</t>
+          <t>syncActivity.phases.autoPreparingTitle</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>phases.discoveringSubtitleSearching</t>
+          <t>phases.autoPreparingTitle</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Searching on the local network</t>
+          <t>Enabling auto-upload…</t>
         </is>
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>正在局域网中搜索</t>
+          <t>正在开启自动同步…</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>正在區域網路中搜尋</t>
+          <t>正在開啟自動同步…</t>
         </is>
       </c>
     </row>
@@ -14071,27 +14069,27 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>syncActivity.phases.discoveringSubtitleWaited</t>
+          <t>syncActivity.phases.defaultTitle</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>phases.discoveringSubtitleWaited</t>
+          <t>phases.defaultTitle</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Waited {{seconds}}s</t>
+          <t>Preparing...</t>
         </is>
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>已等待 {{seconds}} 秒</t>
+          <t>准备中…</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t>已等待 {{seconds}} 秒</t>
+          <t>準備中…</t>
         </is>
       </c>
     </row>
@@ -14103,27 +14101,27 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>syncActivity.phases.discoveringTitle</t>
+          <t>syncActivity.phases.discoveringSubtitleSearching</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>phases.discoveringTitle</t>
+          <t>phases.discoveringSubtitleSearching</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Searching for your computer...</t>
+          <t>Searching on the local network</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>正在搜索电脑…</t>
+          <t>正在局域网中搜索</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t>正在搜尋電腦…</t>
+          <t>正在區域網路中搜尋</t>
         </is>
       </c>
     </row>
@@ -14135,27 +14133,27 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>syncActivity.phases.preparingSubtitle</t>
+          <t>syncActivity.phases.discoveringSubtitleWaited</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>phases.preparingSubtitle</t>
+          <t>phases.discoveringSubtitleWaited</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Establishing a secure connection to your computer</t>
+          <t>Waited {{seconds}}s</t>
         </is>
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>正在与电脑建立安全连接</t>
+          <t>已等待 {{seconds}} 秒</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>正在與電腦建立安全連接</t>
+          <t>已等待 {{seconds}} 秒</t>
         </is>
       </c>
     </row>
@@ -14167,27 +14165,27 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>syncActivity.phases.preparingTitle</t>
+          <t>syncActivity.phases.discoveringTitle</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>phases.preparingTitle</t>
+          <t>phases.discoveringTitle</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Establishing connection...</t>
+          <t>Searching for your computer...</t>
         </is>
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>正在建立连接…</t>
+          <t>正在搜索电脑…</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t>正在建立連接…</t>
+          <t>正在搜尋電腦…</t>
         </is>
       </c>
     </row>
@@ -14199,27 +14197,27 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>syncActivity.phases.reconcilingSubtitle</t>
+          <t>syncActivity.phases.preparingSubtitle</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>phases.reconcilingSubtitle</t>
+          <t>phases.preparingSubtitle</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>First-time setup: verifying previously uploaded files</t>
+          <t>Establishing a secure connection to your computer</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>首次使用需要核对已传文件</t>
+          <t>正在与电脑建立安全连接</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>首次使用需要核對已傳檔案</t>
+          <t>正在與電腦建立安全連接</t>
         </is>
       </c>
     </row>
@@ -14231,27 +14229,27 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>syncActivity.phases.reconcilingTitle</t>
+          <t>syncActivity.phases.preparingTitle</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>phases.reconcilingTitle</t>
+          <t>phases.preparingTitle</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Syncing history...</t>
+          <t>Establishing connection...</t>
         </is>
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>正在同步历史记录…</t>
+          <t>正在建立连接…</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>正在同步歷史記錄…</t>
+          <t>正在建立連接…</t>
         </is>
       </c>
     </row>
@@ -14263,27 +14261,27 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>syncActivity.phases.scanningSubtitleProgress</t>
+          <t>syncActivity.phases.reconcilingSubtitle</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>phases.scanningSubtitleProgress</t>
+          <t>phases.reconcilingSubtitle</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Scanned {{scanned}} / {{total}}</t>
+          <t>First-time setup: verifying previously uploaded files</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>已扫描 {{scanned}} / {{total}} 张</t>
+          <t>首次使用需要核对已传文件</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>已掃描 {{scanned}} / {{total}} 張</t>
+          <t>首次使用需要核對已傳檔案</t>
         </is>
       </c>
     </row>
@@ -14295,27 +14293,27 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>syncActivity.phases.scanningSubtitleReading</t>
+          <t>syncActivity.phases.reconcilingTitle</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>phases.scanningSubtitleReading</t>
+          <t>phases.reconcilingTitle</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Reading photo library</t>
+          <t>Syncing history...</t>
         </is>
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>正在读取相册</t>
+          <t>正在同步历史记录…</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>正在讀取相簿</t>
+          <t>正在同步歷史記錄…</t>
         </is>
       </c>
     </row>
@@ -14327,27 +14325,27 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>syncActivity.phases.scanningTitle</t>
+          <t>syncActivity.phases.scanningSubtitleProgress</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>phases.scanningTitle</t>
+          <t>phases.scanningSubtitleProgress</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Scanning photo library...</t>
+          <t>Scanned {{scanned}} / {{total}}</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>正在扫描相册…</t>
+          <t>已扫描 {{scanned}} / {{total}} 张</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>正在掃描相簿…</t>
+          <t>已掃描 {{scanned}} / {{total}} 張</t>
         </is>
       </c>
     </row>
@@ -14359,27 +14357,27 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>syncActivity.quickEntry.albumDesc</t>
+          <t>syncActivity.phases.scanningSubtitleReading</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>quickEntry.albumDesc</t>
+          <t>phases.scanningSubtitleReading</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Browse and upload photos manually</t>
+          <t>Reading photo library</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>浏览和手动上传素材</t>
+          <t>正在读取相册</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>瀏覽並手動上傳素材</t>
+          <t>正在讀取相簿</t>
         </is>
       </c>
     </row>
@@ -14391,27 +14389,27 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>syncActivity.quickEntry.albumTitle</t>
+          <t>syncActivity.phases.scanningTitle</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>quickEntry.albumTitle</t>
+          <t>phases.scanningTitle</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Album</t>
+          <t>Scanning photo library...</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>相册</t>
+          <t>正在扫描相册…</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t>相簿</t>
+          <t>正在掃描相簿…</t>
         </is>
       </c>
     </row>
@@ -14423,27 +14421,27 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>syncActivity.quickEntry.sharedFilesDesc</t>
+          <t>syncActivity.quickEntry.albumDesc</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>quickEntry.sharedFilesDesc</t>
+          <t>quickEntry.albumDesc</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Browse shared files on your PC</t>
+          <t>Browse and upload photos manually</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>浏览PC设备的共享目录</t>
+          <t>浏览和手动上传素材</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>瀏覽 PC 設備的共享目錄</t>
+          <t>瀏覽並手動上傳素材</t>
         </is>
       </c>
     </row>
@@ -14455,27 +14453,27 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>syncActivity.quickEntry.sharedFilesTitle</t>
+          <t>syncActivity.quickEntry.albumTitle</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>quickEntry.sharedFilesTitle</t>
+          <t>quickEntry.albumTitle</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Shared Files</t>
+          <t>Album</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>共享目录</t>
+          <t>相册</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t>共享目錄</t>
+          <t>相簿</t>
         </is>
       </c>
     </row>
@@ -14487,27 +14485,27 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>syncActivity.quickEntry.title</t>
+          <t>syncActivity.quickEntry.sharedFilesDesc</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>quickEntry.title</t>
+          <t>quickEntry.sharedFilesDesc</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Quick Actions</t>
+          <t>Browse shared files on your PC</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>快捷入口</t>
+          <t>浏览PC设备的共享目录</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t>快捷入口</t>
+          <t>瀏覽 PC 設備的共享目錄</t>
         </is>
       </c>
     </row>
@@ -14519,27 +14517,27 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>syncActivity.running.autoRunningSubtitle</t>
+          <t>syncActivity.quickEntry.sharedFilesTitle</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>running.autoRunningSubtitle</t>
+          <t>quickEntry.sharedFilesTitle</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>New photos will transfer to your PC automatically.</t>
+          <t>Shared Files</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>新素材将自动传输到 PC 端</t>
+          <t>共享目录</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t>新素材將自動傳輸到 PC 端</t>
+          <t>共享目錄</t>
         </is>
       </c>
     </row>
@@ -14551,27 +14549,27 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>syncActivity.running.autoRunningTitle</t>
+          <t>syncActivity.quickEntry.title</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>running.autoRunningTitle</t>
+          <t>quickEntry.title</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Auto Upload Running</t>
+          <t>Quick Actions</t>
         </is>
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>自动上传运行中</t>
+          <t>快捷入口</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>自動上傳執行中</t>
+          <t>快捷入口</t>
         </is>
       </c>
     </row>
@@ -14583,27 +14581,27 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>syncActivity.running.autoTitle</t>
+          <t>syncActivity.running.autoRunningSubtitle</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>running.autoTitle</t>
+          <t>running.autoRunningSubtitle</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Auto Uploading</t>
+          <t>New photos will transfer to your PC automatically.</t>
         </is>
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>正在自动上传</t>
+          <t>新素材将自动传输到 PC 端</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t>正在自動上傳</t>
+          <t>新素材將自動傳輸到 PC 端</t>
         </is>
       </c>
     </row>
@@ -14615,27 +14613,27 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>syncActivity.running.manualTitle</t>
+          <t>syncActivity.running.autoRunningTitle</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>running.manualTitle</t>
+          <t>running.autoRunningTitle</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Manual Upload in Progress</t>
+          <t>Auto Upload Running</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>手动上传中</t>
+          <t>自动上传运行中</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>手動上傳中</t>
+          <t>自動上傳執行中</t>
         </is>
       </c>
     </row>
@@ -14647,27 +14645,27 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>syncActivity.running.queueInfo</t>
+          <t>syncActivity.running.autoTitle</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>running.queueInfo</t>
+          <t>running.autoTitle</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>{{queued}} queued</t>
+          <t>Auto Uploading</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>排队中 {{queued}}项</t>
+          <t>正在自动上传</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>排隊中 {{queued}}項</t>
+          <t>正在自動上傳</t>
         </is>
       </c>
     </row>
@@ -14679,27 +14677,27 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>syncActivity.standby.subtitle</t>
+          <t>syncActivity.running.manualTitle</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>standby.subtitle</t>
+          <t>running.manualTitle</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>New photos will transfer to your PC after you take them.</t>
+          <t>Manual Upload in Progress</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>拍完后会自动传输到 PC 端</t>
+          <t>手动上传中</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>拍完後會自動傳輸到 PC 端</t>
+          <t>手動上傳中</t>
         </is>
       </c>
     </row>
@@ -14711,27 +14709,27 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>syncActivity.standby.title</t>
+          <t>syncActivity.running.queueInfo</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>standby.title</t>
+          <t>running.queueInfo</t>
         </is>
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>Waiting for New Photos</t>
+          <t>{{queued}} queued</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>等待新素材</t>
+          <t>排队中 {{queued}}项</t>
         </is>
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t>等待新素材</t>
+          <t>排隊中 {{queued}}項</t>
         </is>
       </c>
     </row>
@@ -14743,27 +14741,27 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>syncActivity.stats.dataAmount</t>
+          <t>syncActivity.standby.subtitle</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>stats.dataAmount</t>
+          <t>standby.subtitle</t>
         </is>
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>New photos will transfer to your PC after you take them.</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>数据量</t>
+          <t>拍完后会自动传输到 PC 端</t>
         </is>
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>資料量</t>
+          <t>拍完後會自動傳輸到 PC 端</t>
         </is>
       </c>
     </row>
@@ -14775,27 +14773,27 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>syncActivity.stats.progress</t>
+          <t>syncActivity.standby.title</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>stats.progress</t>
+          <t>standby.title</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>Progress</t>
+          <t>Waiting for New Photos</t>
         </is>
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t>进度</t>
+          <t>等待新素材</t>
         </is>
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t>進度</t>
+          <t>等待新素材</t>
         </is>
       </c>
     </row>
@@ -14807,27 +14805,27 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>syncActivity.stats.speed</t>
+          <t>syncActivity.stats.dataAmount</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>stats.speed</t>
+          <t>stats.dataAmount</t>
         </is>
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>速度</t>
+          <t>数据量</t>
         </is>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>速度</t>
+          <t>資料量</t>
         </is>
       </c>
     </row>
@@ -14839,27 +14837,27 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>syncActivity.stats.transferred</t>
+          <t>syncActivity.stats.progress</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>stats.transferred</t>
+          <t>stats.progress</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Transferred</t>
+          <t>Progress</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>已传输</t>
+          <t>进度</t>
         </is>
       </c>
       <c r="F450" t="inlineStr">
         <is>
-          <t>已傳輸</t>
+          <t>進度</t>
         </is>
       </c>
     </row>
@@ -14871,27 +14869,27 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>syncActivity.stats.transferredCount</t>
+          <t>syncActivity.stats.speed</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>stats.transferredCount</t>
+          <t>stats.speed</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>{{count}}</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>{{count}} 个</t>
+          <t>速度</t>
         </is>
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>{{count}} 個</t>
+          <t>速度</t>
         </is>
       </c>
     </row>
@@ -14903,91 +14901,91 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>syncActivity.title</t>
+          <t>syncActivity.stats.transferred</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>stats.transferred</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>Sync Activity</t>
+          <t>Transferred</t>
         </is>
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>同步动态</t>
+          <t>已传输</t>
         </is>
       </c>
       <c r="F452" t="inlineStr">
         <is>
-          <t>同步動態</t>
+          <t>已傳輸</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>syncStatus</t>
+          <t>syncActivity</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>syncStatus.banners.connecting</t>
+          <t>syncActivity.stats.transferredCount</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>banners.connecting</t>
+          <t>stats.transferredCount</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>Connecting to "{{device}}".</t>
+          <t>{{count}}</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>正在连接到"{{device}}"。</t>
+          <t>{{count}} 个</t>
         </is>
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>正在連接到"{{device}}"。</t>
+          <t>{{count}} 個</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>syncStatus</t>
+          <t>syncActivity</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>syncStatus.banners.connectingAutoResume</t>
+          <t>syncActivity.title</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>banners.connectingAutoResume</t>
+          <t>title</t>
         </is>
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>Sync will resume automatically once connected.</t>
+          <t>Sync Activity</t>
         </is>
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>连接建立后会自动继续当前同步任务。</t>
+          <t>同步动态</t>
         </is>
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>連接建立後會自動繼續當前同步任務。</t>
+          <t>同步動態</t>
         </is>
       </c>
     </row>
@@ -14999,27 +14997,27 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>syncStatus.banners.connectionErrorResume</t>
+          <t>syncStatus.banners.connecting</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>banners.connectionErrorResume</t>
+          <t>banners.connecting</t>
         </is>
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>Sync will resume when the network is restored or Vivi Drop is reopened on your computer.</t>
+          <t>Connecting to "{{device}}".</t>
         </is>
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>恢复网络或重新打开电脑端 Vivi Drop 后会自动继续。</t>
+          <t>正在连接到"{{device}}"。</t>
         </is>
       </c>
       <c r="F455" t="inlineStr">
         <is>
-          <t>恢復網路或重新打開電腦端 Vivi Drop 後會自動繼續。</t>
+          <t>正在連接到"{{device}}"。</t>
         </is>
       </c>
     </row>
@@ -15031,27 +15029,27 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>syncStatus.banners.networkAutoResume</t>
+          <t>syncStatus.banners.connectingAutoResume</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>banners.networkAutoResume</t>
+          <t>banners.connectingAutoResume</t>
         </is>
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>Progress saved ({{transferred}} / {{total}}). Sync will resume when the network recovers.</t>
+          <t>Sync will resume automatically once connected.</t>
         </is>
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t>已保留当前进度 {{transferred}} / {{total}}，网络恢复后会自动继续。</t>
+          <t>连接建立后会自动继续当前同步任务。</t>
         </is>
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>已保留當前進度 {{transferred}} / {{total}}，網路恢復後會自動繼續。</t>
+          <t>連接建立後會自動繼續當前同步任務。</t>
         </is>
       </c>
     </row>
@@ -15063,27 +15061,27 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>syncStatus.banners.networkPaused</t>
+          <t>syncStatus.banners.connectionErrorResume</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>banners.networkPaused</t>
+          <t>banners.connectionErrorResume</t>
         </is>
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>Transfer paused — waiting for the network to recover.</t>
+          <t>Sync will resume when the network is restored or Vivi Drop is reopened on your computer.</t>
         </is>
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>传输已暂停，等待网络恢复。</t>
+          <t>恢复网络或重新打开电脑端 Vivi Drop 后会自动继续。</t>
         </is>
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t>傳輸已暫停，等待網路恢復。</t>
+          <t>恢復網路或重新打開電腦端 Vivi Drop 後會自動繼續。</t>
         </is>
       </c>
     </row>
@@ -15095,27 +15093,27 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>syncStatus.banners.networkReconnecting</t>
+          <t>syncStatus.banners.networkAutoResume</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>banners.networkReconnecting</t>
+          <t>banners.networkAutoResume</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>Network hiccup — reconnecting to "{{device}}".</t>
+          <t>Progress saved ({{transferred}} / {{total}}). Sync will resume when the network recovers.</t>
         </is>
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>网络波动，正在重连"{{device}}"。</t>
+          <t>已保留当前进度 {{transferred}} / {{total}}，网络恢复后会自动继续。</t>
         </is>
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>網路波動，正在重連"{{device}}"。</t>
+          <t>已保留當前進度 {{transferred}} / {{total}}，網路恢復後會自動繼續。</t>
         </is>
       </c>
     </row>
@@ -15127,27 +15125,27 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>syncStatus.banners.networkWithRetry</t>
+          <t>syncStatus.banners.networkPaused</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>banners.networkWithRetry</t>
+          <t>banners.networkPaused</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>Progress saved ({{transferred}} / {{total}}). Retry {{attempt}} in {{seconds}}s after the network recovers.</t>
+          <t>Transfer paused — waiting for the network to recover.</t>
         </is>
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>已保留当前进度 {{transferred}} / {{total}}，网络恢复后将在 {{seconds}} 秒后发起第 {{attempt}} 次重试。</t>
+          <t>传输已暂停，等待网络恢复。</t>
         </is>
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t>已保留當前進度 {{transferred}} / {{total}}，網路恢復後將在 {{seconds}} 秒後發起第 {{attempt}} 次重試。</t>
+          <t>傳輸已暫停，等待網路恢復。</t>
         </is>
       </c>
     </row>
@@ -15159,27 +15157,27 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>syncStatus.banners.notConnected</t>
+          <t>syncStatus.banners.networkReconnecting</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>banners.notConnected</t>
+          <t>banners.networkReconnecting</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>Not connected to "{{device}}" — make sure Vivi Drop is running on your computer.</t>
+          <t>Network hiccup — reconnecting to "{{device}}".</t>
         </is>
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>未连接到"{{device}}"，请确认电脑端 Vivi Drop 正在运行。</t>
+          <t>网络波动，正在重连"{{device}}"。</t>
         </is>
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>未連接到"{{device}}"，請確認電腦端 Vivi Drop 正在運行。</t>
+          <t>網路波動，正在重連"{{device}}"。</t>
         </is>
       </c>
     </row>
@@ -15191,27 +15189,27 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>syncStatus.banners.permissionDetail</t>
+          <t>syncStatus.banners.networkWithRetry</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>banners.permissionDetail</t>
+          <t>banners.networkWithRetry</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>Allow access in system settings — sync will resume automatically.</t>
+          <t>Progress saved ({{transferred}} / {{total}}). Retry {{attempt}} in {{seconds}}s after the network recovers.</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>打开系统设置后允许访问照片，恢复后会自动继续同步。</t>
+          <t>已保留当前进度 {{transferred}} / {{total}}，网络恢复后将在 {{seconds}} 秒后发起第 {{attempt}} 次重试。</t>
         </is>
       </c>
       <c r="F461" t="inlineStr">
         <is>
-          <t>開啟系統設定後允許存取照片，恢復後會自動繼續同步。</t>
+          <t>已保留當前進度 {{transferred}} / {{total}}，網路恢復後將在 {{seconds}} 秒後發起第 {{attempt}} 次重試。</t>
         </is>
       </c>
     </row>
@@ -15223,27 +15221,27 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>syncStatus.banners.permissionRequired</t>
+          <t>syncStatus.banners.notConnected</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>banners.permissionRequired</t>
+          <t>banners.notConnected</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>Photo library access is required.</t>
+          <t>Not connected to "{{device}}" — make sure Vivi Drop is running on your computer.</t>
         </is>
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>需要授予照片访问权限。</t>
+          <t>未连接到"{{device}}"，请确认电脑端 Vivi Drop 正在运行。</t>
         </is>
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>需要授予照片存取權限。</t>
+          <t>未連接到"{{device}}"，請確認電腦端 Vivi Drop 正在運行。</t>
         </is>
       </c>
     </row>
@@ -15255,27 +15253,27 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>syncStatus.banners.progressWindowsNoRetry</t>
+          <t>syncStatus.banners.permissionDetail</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>banners.progressWindowsNoRetry</t>
+          <t>banners.permissionDetail</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>Progress saved ({{transferred}} / {{total}}). Check firewall, security software, or VPN on this Windows PC — sync will resume automatically.</t>
+          <t>Allow access in system settings — sync will resume automatically.</t>
         </is>
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>已保留当前进度 {{transferred}} / {{total}}，请检查这台 Windows 电脑上的防火墙、安全软件或 VPN，处理后会自动继续。</t>
+          <t>打开系统设置后允许访问照片，恢复后会自动继续同步。</t>
         </is>
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>已保留當前進度 {{transferred}} / {{total}}，請檢查這台 Windows 電腦上的防火牆、安全軟體或 VPN，處理後會自動繼續。</t>
+          <t>開啟系統設定後允許存取照片，恢復後會自動繼續同步。</t>
         </is>
       </c>
     </row>
@@ -15287,27 +15285,27 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>syncStatus.banners.progressWindowsRetry</t>
+          <t>syncStatus.banners.permissionRequired</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>banners.progressWindowsRetry</t>
+          <t>banners.permissionRequired</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t>Progress saved ({{transferred}} / {{total}}). Retry {{attempt}} in {{seconds}}s. Check firewall, security software, or VPN on this Windows PC.</t>
+          <t>Photo library access is required.</t>
         </is>
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>已保留当前进度 {{transferred}} / {{total}}，将在 {{seconds}} 秒后发起第 {{attempt}} 次重试。请检查这台 Windows 电脑上的防火墙、安全软件或 VPN。</t>
+          <t>需要授予照片访问权限。</t>
         </is>
       </c>
       <c r="F464" t="inlineStr">
         <is>
-          <t>已保留當前進度 {{transferred}} / {{total}}，將在 {{seconds}} 秒後發起第 {{attempt}} 次重試。請檢查這台 Windows 電腦上的防火牆、安全軟體或 VPN。</t>
+          <t>需要授予照片存取權限。</t>
         </is>
       </c>
     </row>
@@ -15319,27 +15317,27 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>syncStatus.banners.progressWithRetry</t>
+          <t>syncStatus.banners.progressWindowsNoRetry</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>banners.progressWithRetry</t>
+          <t>banners.progressWindowsNoRetry</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>Progress saved ({{transferred}} / {{total}}). Retry {{attempt}} in {{seconds}}s.</t>
+          <t>Progress saved ({{transferred}} / {{total}}). Check firewall, security software, or VPN on this Windows PC — sync will resume automatically.</t>
         </is>
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>已保留当前进度 {{transferred}} / {{total}}，将在 {{seconds}} 秒后发起第 {{attempt}} 次重试。</t>
+          <t>已保留当前进度 {{transferred}} / {{total}}，请检查这台 Windows 电脑上的防火墙、安全软件或 VPN，处理后会自动继续。</t>
         </is>
       </c>
       <c r="F465" t="inlineStr">
         <is>
-          <t>已保留當前進度 {{transferred}} / {{total}}，將在 {{seconds}} 秒後發起第 {{attempt}} 次重試。</t>
+          <t>已保留當前進度 {{transferred}} / {{total}}，請檢查這台 Windows 電腦上的防火牆、安全軟體或 VPN，處理後會自動繼續。</t>
         </is>
       </c>
     </row>
@@ -15351,27 +15349,27 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>syncStatus.banners.retryingReconnect</t>
+          <t>syncStatus.banners.progressWindowsRetry</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>banners.retryingReconnect</t>
+          <t>banners.progressWindowsRetry</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>Progress saved ({{transferred}} / {{total}}). Reconnecting...</t>
+          <t>Progress saved ({{transferred}} / {{total}}). Retry {{attempt}} in {{seconds}}s. Check firewall, security software, or VPN on this Windows PC.</t>
         </is>
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>已保留当前进度 {{transferred}} / {{total}}，正在重新建立连接。</t>
+          <t>已保留当前进度 {{transferred}} / {{total}}，将在 {{seconds}} 秒后发起第 {{attempt}} 次重试。请检查这台 Windows 电脑上的防火墙、安全软件或 VPN。</t>
         </is>
       </c>
       <c r="F466" t="inlineStr">
         <is>
-          <t>已保留當前進度 {{transferred}} / {{total}}，正在重新建立連接。</t>
+          <t>已保留當前進度 {{transferred}} / {{total}}，將在 {{seconds}} 秒後發起第 {{attempt}} 次重試。請檢查這台 Windows 電腦上的防火牆、安全軟體或 VPN。</t>
         </is>
       </c>
     </row>
@@ -15383,27 +15381,27 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>syncStatus.banners.windowsInterrupted</t>
+          <t>syncStatus.banners.progressWithRetry</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>banners.windowsInterrupted</t>
+          <t>banners.progressWithRetry</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>"{{device}}" interrupted the transfer.</t>
+          <t>Progress saved ({{transferred}} / {{total}}). Retry {{attempt}} in {{seconds}}s.</t>
         </is>
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>"{{device}}"中断了传输连接。</t>
+          <t>已保留当前进度 {{transferred}} / {{total}}，将在 {{seconds}} 秒后发起第 {{attempt}} 次重试。</t>
         </is>
       </c>
       <c r="F467" t="inlineStr">
         <is>
-          <t>"{{device}}"中斷了傳輸連接。</t>
+          <t>已保留當前進度 {{transferred}} / {{total}}，將在 {{seconds}} 秒後發起第 {{attempt}} 次重試。</t>
         </is>
       </c>
     </row>
@@ -15415,27 +15413,27 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>syncStatus.completion.filesUnit</t>
+          <t>syncStatus.banners.retryingReconnect</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>completion.filesUnit</t>
+          <t>banners.retryingReconnect</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>files</t>
+          <t>Progress saved ({{transferred}} / {{total}}). Reconnecting...</t>
         </is>
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>个文件</t>
+          <t>已保留当前进度 {{transferred}} / {{total}}，正在重新建立连接。</t>
         </is>
       </c>
       <c r="F468" t="inlineStr">
         <is>
-          <t>個檔案</t>
+          <t>已保留當前進度 {{transferred}} / {{total}}，正在重新建立連接。</t>
         </is>
       </c>
     </row>
@@ -15447,27 +15445,27 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>syncStatus.completion.latestSync</t>
+          <t>syncStatus.banners.windowsInterrupted</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>completion.latestSync</t>
+          <t>banners.windowsInterrupted</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>Last successful sync: {{label}}</t>
+          <t>"{{device}}" interrupted the transfer.</t>
         </is>
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>最近一次成功同步：{{label}}</t>
+          <t>"{{device}}"中断了传输连接。</t>
         </is>
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t>最近一次成功同步：{{label}}</t>
+          <t>"{{device}}"中斷了傳輸連接。</t>
         </is>
       </c>
     </row>
@@ -15479,27 +15477,27 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>syncStatus.completion.subtitle</t>
+          <t>syncStatus.completion.filesUnit</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>completion.subtitle</t>
+          <t>completion.filesUnit</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>This sync is complete.</t>
+          <t>files</t>
         </is>
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>本次同步已全部完成</t>
+          <t>个文件</t>
         </is>
       </c>
       <c r="F470" t="inlineStr">
         <is>
-          <t>本次同步已全部完成</t>
+          <t>個檔案</t>
         </is>
       </c>
     </row>
@@ -15511,27 +15509,27 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>syncStatus.completion.title</t>
+          <t>syncStatus.completion.latestSync</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>completion.title</t>
+          <t>completion.latestSync</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>All Files Synced</t>
+          <t>Last successful sync: {{label}}</t>
         </is>
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>所有文件已同步</t>
+          <t>最近一次成功同步：{{label}}</t>
         </is>
       </c>
       <c r="F471" t="inlineStr">
         <is>
-          <t>所有檔案已同步</t>
+          <t>最近一次成功同步：{{label}}</t>
         </is>
       </c>
     </row>
@@ -15543,27 +15541,27 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>syncStatus.phases.cloudDownloading</t>
+          <t>syncStatus.completion.subtitle</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>phases.cloudDownloading</t>
+          <t>completion.subtitle</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
         <is>
-          <t>Preparing media</t>
+          <t>This sync is complete.</t>
         </is>
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>准备素材中</t>
+          <t>本次同步已全部完成</t>
         </is>
       </c>
       <c r="F472" t="inlineStr">
         <is>
-          <t>準備素材中</t>
+          <t>本次同步已全部完成</t>
         </is>
       </c>
     </row>
@@ -15575,27 +15573,27 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>syncStatus.phases.default</t>
+          <t>syncStatus.completion.title</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>phases.default</t>
+          <t>completion.title</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
         <is>
-          <t>Sync summary</t>
+          <t>All Files Synced</t>
         </is>
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>同步摘要</t>
+          <t>所有文件已同步</t>
         </is>
       </c>
       <c r="F473" t="inlineStr">
         <is>
-          <t>同步摘要</t>
+          <t>所有檔案已同步</t>
         </is>
       </c>
     </row>
@@ -15607,27 +15605,27 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>syncStatus.phases.pausedNoPermission</t>
+          <t>syncStatus.phases.cloudDownloading</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>phases.pausedNoPermission</t>
+          <t>phases.cloudDownloading</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
         <is>
-          <t>Waiting for permission</t>
+          <t>Preparing media</t>
         </is>
       </c>
       <c r="E474" t="inlineStr">
         <is>
-          <t>等待权限</t>
+          <t>准备素材中</t>
         </is>
       </c>
       <c r="F474" t="inlineStr">
         <is>
-          <t>等待權限</t>
+          <t>準備素材中</t>
         </is>
       </c>
     </row>
@@ -15639,27 +15637,27 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>syncStatus.phases.preparing</t>
+          <t>syncStatus.phases.default</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>phases.preparing</t>
+          <t>phases.default</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>Preparing sync</t>
+          <t>Sync summary</t>
         </is>
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>准备同步</t>
+          <t>同步摘要</t>
         </is>
       </c>
       <c r="F475" t="inlineStr">
         <is>
-          <t>準備同步</t>
+          <t>同步摘要</t>
         </is>
       </c>
     </row>
@@ -15671,27 +15669,27 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>syncStatus.phases.reconnecting</t>
+          <t>syncStatus.phases.pausedNoPermission</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>phases.reconnecting</t>
+          <t>phases.pausedNoPermission</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
         <is>
-          <t>Waiting to reconnect</t>
+          <t>Waiting for permission</t>
         </is>
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>等待重连</t>
+          <t>等待权限</t>
         </is>
       </c>
       <c r="F476" t="inlineStr">
         <is>
-          <t>等待重連</t>
+          <t>等待權限</t>
         </is>
       </c>
     </row>
@@ -15703,27 +15701,27 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>syncStatus.phases.uploading</t>
+          <t>syncStatus.phases.preparing</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>phases.uploading</t>
+          <t>phases.preparing</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>Syncing</t>
+          <t>Preparing sync</t>
         </is>
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>正在同步</t>
+          <t>准备同步</t>
         </is>
       </c>
       <c r="F477" t="inlineStr">
         <is>
-          <t>正在同步</t>
+          <t>準備同步</t>
         </is>
       </c>
     </row>
@@ -15735,27 +15733,27 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>syncStatus.queue.itemStatus.cloudDownloading</t>
+          <t>syncStatus.phases.reconnecting</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>queue.itemStatus.cloudDownloading</t>
+          <t>phases.reconnecting</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>Downloading iCloud original</t>
+          <t>Waiting to reconnect</t>
         </is>
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>下载 iCloud 原件中</t>
+          <t>等待重连</t>
         </is>
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>下載 iCloud 原件中</t>
+          <t>等待重連</t>
         </is>
       </c>
     </row>
@@ -15767,27 +15765,27 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>syncStatus.queue.itemStatus.preparing</t>
+          <t>syncStatus.phases.uploading</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>queue.itemStatus.preparing</t>
+          <t>phases.uploading</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>Preparing</t>
+          <t>Syncing</t>
         </is>
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>准备中</t>
+          <t>正在同步</t>
         </is>
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t>準備中</t>
+          <t>正在同步</t>
         </is>
       </c>
     </row>
@@ -15799,27 +15797,27 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>syncStatus.queue.itemStatus.transferring</t>
+          <t>syncStatus.queue.itemStatus.cloudDownloading</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>queue.itemStatus.transferring</t>
+          <t>queue.itemStatus.cloudDownloading</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>Transferring {{percent}}%</t>
+          <t>Downloading iCloud original</t>
         </is>
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>传输中 {{percent}}%</t>
+          <t>下载 iCloud 原件中</t>
         </is>
       </c>
       <c r="F480" t="inlineStr">
         <is>
-          <t>傳輸中 {{percent}}%</t>
+          <t>下載 iCloud 原件中</t>
         </is>
       </c>
     </row>
@@ -15831,27 +15829,27 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>syncStatus.queue.itemStatus.uploading</t>
+          <t>syncStatus.queue.itemStatus.preparing</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>queue.itemStatus.uploading</t>
+          <t>queue.itemStatus.preparing</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>Transferring</t>
+          <t>Preparing</t>
         </is>
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>传输中</t>
+          <t>准备中</t>
         </is>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>傳輸中</t>
+          <t>準備中</t>
         </is>
       </c>
     </row>
@@ -15863,27 +15861,27 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>syncStatus.summary.currentFile</t>
+          <t>syncStatus.queue.itemStatus.transferring</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>summary.currentFile</t>
+          <t>queue.itemStatus.transferring</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>Current file: {{name}}</t>
+          <t>Transferring {{percent}}%</t>
         </is>
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>当前文件：{{name}}</t>
+          <t>传输中 {{percent}}%</t>
         </is>
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>當前檔案：{{name}}</t>
+          <t>傳輸中 {{percent}}%</t>
         </is>
       </c>
     </row>
@@ -15895,27 +15893,27 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>syncStatus.summary.filesCompleted</t>
+          <t>syncStatus.queue.itemStatus.uploading</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>summary.filesCompleted</t>
+          <t>queue.itemStatus.uploading</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>{{completed}} / {{total}} files done</t>
+          <t>Transferring</t>
         </is>
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>{{completed}} / {{total}} 个文件已完成</t>
+          <t>传输中</t>
         </is>
       </c>
       <c r="F483" t="inlineStr">
         <is>
-          <t>{{completed}} / {{total}} 個檔案已完成</t>
+          <t>傳輸中</t>
         </is>
       </c>
     </row>
@@ -15927,27 +15925,27 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>syncStatus.summary.speed</t>
+          <t>syncStatus.summary.currentFile</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>summary.speed</t>
+          <t>summary.currentFile</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Current file: {{name}}</t>
         </is>
       </c>
       <c r="E484" t="inlineStr">
         <is>
-          <t>当前速度</t>
+          <t>当前文件：{{name}}</t>
         </is>
       </c>
       <c r="F484" t="inlineStr">
         <is>
-          <t>當前速度</t>
+          <t>當前檔案：{{name}}</t>
         </is>
       </c>
     </row>
@@ -15959,25 +15957,89 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
+          <t>syncStatus.summary.filesCompleted</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>summary.filesCompleted</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>{{completed}} / {{total}} files done</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>{{completed}} / {{total}} 个文件已完成</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>{{completed}} / {{total}} 個檔案已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>syncStatus</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>syncStatus.summary.speed</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>summary.speed</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>当前速度</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>當前速度</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>syncStatus</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
           <t>syncStatus.summary.transferred</t>
         </is>
       </c>
-      <c r="C485" t="inlineStr">
+      <c r="C487" t="inlineStr">
         <is>
           <t>summary.transferred</t>
         </is>
       </c>
-      <c r="D485" t="inlineStr">
+      <c r="D487" t="inlineStr">
         <is>
           <t>Transferred</t>
         </is>
       </c>
-      <c r="E485" t="inlineStr">
+      <c r="E487" t="inlineStr">
         <is>
           <t>已传输</t>
         </is>
       </c>
-      <c r="F485" t="inlineStr">
+      <c r="F487" t="inlineStr">
         <is>
           <t>已傳輸</t>
         </is>

</xml_diff>